<commit_message>
Fixed time tracking and cell color
</commit_message>
<xml_diff>
--- a/session_data_2025-05-20.xlsx
+++ b/session_data_2025-05-20.xlsx
@@ -26,7 +26,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -43,11 +43,6 @@
         <fgColor rgb="FFF0E68C"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFADD8E6"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -61,11 +56,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,17 +476,17 @@
           <t>00:01</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>2025-05-20 21:09:12</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2025-05-20 21:10:49</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
+          <t>2025-05-20 21:48:54</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>Browser</t>
         </is>
@@ -511,54 +505,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>00:03</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
+          <t>02:24</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>2025-05-20 21:09:03</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2025-05-20 21:13:38</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
+          <t>2025-05-20 21:49:00</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Work</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Друзья - Discord</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Discord</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>2025-05-20 21:12:40</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2025-05-20 21:13:37</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Messenger</t>
         </is>
       </c>
     </row>

</xml_diff>